<commit_message>
Fixtures: regional price strengths so a split award beats a single award
</commit_message>
<xml_diff>
--- a/data/vendor_docs/vendor-A-excel-ignores-template.xlsx
+++ b/data/vendor_docs/vendor-A-excel-ignores-template.xlsx
@@ -584,7 +584,7 @@
         <v>20GP</v>
       </c>
       <c r="E9">
-        <v>36200</v>
+        <v>37500</v>
       </c>
       <c r="F9">
         <v>12</v>
@@ -607,7 +607,7 @@
         <v>40HC</v>
       </c>
       <c r="E10">
-        <v>53900</v>
+        <v>56200</v>
       </c>
       <c r="F10">
         <v>12</v>
@@ -630,7 +630,7 @@
         <v>40HC</v>
       </c>
       <c r="E11">
-        <v>155000</v>
+        <v>161000</v>
       </c>
       <c r="F11">
         <v>26</v>
@@ -653,7 +653,7 @@
         <v>40HC</v>
       </c>
       <c r="E12">
-        <v>152500</v>
+        <v>158500</v>
       </c>
       <c r="F12">
         <v>27</v>
@@ -676,7 +676,7 @@
         <v>40HC</v>
       </c>
       <c r="E13">
-        <v>222000</v>
+        <v>231000</v>
       </c>
       <c r="F13">
         <v>34</v>
@@ -745,7 +745,7 @@
         <v>40HC</v>
       </c>
       <c r="E16">
-        <v>159500</v>
+        <v>166000</v>
       </c>
       <c r="F16">
         <v>28</v>
@@ -768,7 +768,7 @@
         <v>40HC</v>
       </c>
       <c r="E17">
-        <v>163000</v>
+        <v>169500</v>
       </c>
       <c r="F17">
         <v>27</v>
@@ -791,7 +791,7 @@
         <v>20GP</v>
       </c>
       <c r="E18">
-        <v>21500</v>
+        <v>22100</v>
       </c>
       <c r="F18">
         <v>4</v>
@@ -975,7 +975,7 @@
         <v>LCL per CBM</v>
       </c>
       <c r="E26">
-        <v>3820</v>
+        <v>4050</v>
       </c>
       <c r="F26">
         <v>30</v>
@@ -998,7 +998,7 @@
         <v>LCL per CBM</v>
       </c>
       <c r="E27">
-        <v>5250</v>
+        <v>5600</v>
       </c>
       <c r="F27">
         <v>38</v>
@@ -1021,7 +1021,7 @@
         <v>LCL per CBM</v>
       </c>
       <c r="E28">
-        <v>3700</v>
+        <v>3950</v>
       </c>
       <c r="F28">
         <v>32</v>
@@ -1090,7 +1090,7 @@
         <v>Air per kg chargeable</v>
       </c>
       <c r="E31">
-        <v>121</v>
+        <v>126</v>
       </c>
       <c r="F31">
         <v>2</v>

</xml_diff>